<commit_message>
Ajustement tailles images messages institutionnels
</commit_message>
<xml_diff>
--- a/BD_Global.xlsx
+++ b/BD_Global.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\UltraBook 3.1\Desktop\STREAMLIT - IMPORTSUBSTITUTION\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{645D29A2-3E2A-4E76-9E8F-972FCBC97D91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF51B57E-79EF-4836-BF03-4899BF6A295F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1520" yWindow="0" windowWidth="15660" windowHeight="10080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -76,18 +76,19 @@
     <t>cible_piisah_production</t>
   </si>
   <si>
-    <t>Taux de couverture</t>
+    <t>Taux de contenu local</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="#,##0."/>
     <numFmt numFmtId="165" formatCode="_-* #,##0\ _€_-;\-* #,##0\ _€_-;_-* &quot;-&quot;??\ _€_-;_-@_-"/>
     <numFmt numFmtId="166" formatCode="#,##0.."/>
+    <numFmt numFmtId="173" formatCode="_-* #,##0.0000000\ _€_-;\-* #,##0.0000000\ _€_-;_-* &quot;-&quot;??\ _€_-;_-@_-"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -234,7 +235,7 @@
     <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="173" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Milliers" xfId="1" builtinId="3"/>
@@ -516,6 +517,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="14.5"/>
   <cols>
     <col min="2" max="2" width="12.81640625"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
     <col min="5" max="7" width="11.90625"/>
     <col min="9" max="14" width="12.81640625"/>
     <col min="15" max="15" width="12.54296875" customWidth="1"/>
@@ -1494,7 +1496,7 @@
         <v>0.40915878546540568</v>
       </c>
       <c r="C23">
-        <f t="shared" ref="C9:C71" si="3">E23/(E23+F23)</f>
+        <f t="shared" ref="C23:C71" si="3">E23/(E23+F23)</f>
         <v>0.59084121453459437</v>
       </c>
       <c r="D23" s="3">
@@ -2115,17 +2117,17 @@
       </c>
       <c r="B38">
         <f t="shared" si="0"/>
-        <v>0.98701941377997715</v>
+        <v>0.98702354672973502</v>
       </c>
       <c r="C38">
         <f t="shared" si="3"/>
-        <v>1.2980586220022839E-2</v>
+        <v>1.2976453270264931E-2</v>
       </c>
       <c r="D38" s="3">
         <v>2021</v>
       </c>
       <c r="E38" s="4">
-        <v>34100</v>
+        <v>34089</v>
       </c>
       <c r="F38" s="4">
         <v>2592900</v>
@@ -2150,17 +2152,17 @@
       </c>
       <c r="B39">
         <f t="shared" si="0"/>
-        <v>0.82558810138108973</v>
+        <v>0.99555060364794867</v>
       </c>
       <c r="C39">
         <f t="shared" si="3"/>
-        <v>0.17441189861891029</v>
+        <v>4.4493963520513486E-3</v>
       </c>
       <c r="D39" s="3">
         <v>2022</v>
       </c>
       <c r="E39" s="4">
-        <v>574600</v>
+        <v>12156</v>
       </c>
       <c r="F39" s="4">
         <v>2719900</v>
@@ -2220,17 +2222,17 @@
       </c>
       <c r="B41">
         <f t="shared" si="0"/>
-        <v>0.84111503078093652</v>
+        <v>0.97811783102370975</v>
       </c>
       <c r="C41">
         <f t="shared" si="3"/>
-        <v>0.15888496921906342</v>
+        <v>2.1882168976290296E-2</v>
       </c>
       <c r="D41" s="3">
         <v>2024</v>
       </c>
       <c r="E41" s="4">
-        <v>689100</v>
+        <v>81612</v>
       </c>
       <c r="F41" s="4">
         <v>3648000</v>
@@ -2624,17 +2626,17 @@
       </c>
       <c r="B52">
         <f t="shared" si="0"/>
-        <v>3.9142119728080907E-4</v>
+        <v>0.28138951732784839</v>
       </c>
       <c r="C52">
         <f t="shared" si="3"/>
-        <v>0.99960857880271914</v>
+        <v>0.71861048267215155</v>
       </c>
       <c r="D52" s="5">
         <v>2015</v>
       </c>
       <c r="E52" s="10">
-        <v>707247338</v>
+        <v>707247.33799999999</v>
       </c>
       <c r="F52" s="6">
         <v>276940</v>
@@ -2667,17 +2669,17 @@
       </c>
       <c r="B53">
         <f t="shared" si="0"/>
-        <v>5.8448883839491499E-4</v>
+        <v>0.36901776206282089</v>
       </c>
       <c r="C53" s="20">
         <f>E53/(E53+F53)</f>
-        <v>0.9994155111616051</v>
+        <v>0.63098223793717911</v>
       </c>
       <c r="D53" s="5">
         <v>2016</v>
       </c>
       <c r="E53" s="10">
-        <v>614400067</v>
+        <v>614400.06700000004</v>
       </c>
       <c r="F53" s="11">
         <v>359320</v>
@@ -2710,17 +2712,17 @@
       </c>
       <c r="B54">
         <f t="shared" si="0"/>
-        <v>3.968796664389008E-4</v>
+        <v>0.28419946897889475</v>
       </c>
       <c r="C54">
         <f t="shared" si="3"/>
-        <v>0.99960312033356113</v>
+        <v>0.71580053102110519</v>
       </c>
       <c r="D54" s="5">
         <v>2017</v>
       </c>
       <c r="E54" s="10">
-        <v>728443000</v>
+        <v>728443</v>
       </c>
       <c r="F54" s="11">
         <v>289219</v>
@@ -2753,17 +2755,17 @@
       </c>
       <c r="B55">
         <f t="shared" si="0"/>
-        <v>5.8989380368617086E-4</v>
+        <v>0.37116488546849946</v>
       </c>
       <c r="C55">
         <f t="shared" si="3"/>
-        <v>0.99941010619631376</v>
+        <v>0.62883511453150054</v>
       </c>
       <c r="D55" s="5">
         <v>2018</v>
       </c>
       <c r="E55" s="10">
-        <v>561112000</v>
+        <v>561112</v>
       </c>
       <c r="F55" s="11">
         <v>331191.86</v>
@@ -2796,17 +2798,17 @@
       </c>
       <c r="B56">
         <f t="shared" si="0"/>
-        <v>3.3244106448174969E-4</v>
+        <v>0.24956002734141619</v>
       </c>
       <c r="C56">
         <f t="shared" si="3"/>
-        <v>0.99966755893551817</v>
+        <v>0.75043997265858375</v>
       </c>
       <c r="D56" s="5">
         <v>2019</v>
       </c>
       <c r="E56" s="10">
-        <v>894485799</v>
+        <v>894485.799</v>
       </c>
       <c r="F56" s="11">
         <v>297462.7</v>
@@ -2839,17 +2841,17 @@
       </c>
       <c r="B57">
         <f t="shared" si="0"/>
-        <v>4.8373048233534249E-4</v>
+        <v>0.32612947355591526</v>
       </c>
       <c r="C57">
         <f t="shared" si="3"/>
-        <v>0.9995162695176647</v>
+        <v>0.67387052644408474</v>
       </c>
       <c r="D57" s="5">
         <v>2020</v>
       </c>
       <c r="E57" s="10">
-        <v>591597000</v>
+        <v>591597</v>
       </c>
       <c r="F57" s="11">
         <v>286312</v>
@@ -2882,17 +2884,17 @@
       </c>
       <c r="B58">
         <f t="shared" si="0"/>
-        <v>4.5562470394824617E-4</v>
+        <v>0.31310774153121945</v>
       </c>
       <c r="C58">
         <f t="shared" si="3"/>
-        <v>0.99954437529605178</v>
+        <v>0.68689225846878066</v>
       </c>
       <c r="D58" s="5">
         <v>2021</v>
       </c>
       <c r="E58" s="12">
-        <v>776601237.35300004</v>
+        <v>776601.23735299997</v>
       </c>
       <c r="F58" s="11">
         <v>354000</v>
@@ -2925,17 +2927,17 @@
       </c>
       <c r="B59">
         <f t="shared" si="0"/>
-        <v>4.0389458340782527E-4</v>
+        <v>0.28777859847872078</v>
       </c>
       <c r="C59">
         <f t="shared" si="3"/>
-        <v>0.99959610541659216</v>
+        <v>0.71222140152127911</v>
       </c>
       <c r="D59" s="5">
         <v>2022</v>
       </c>
       <c r="E59" s="12">
-        <v>841463812.10186005</v>
+        <v>841463.81210185995</v>
       </c>
       <c r="F59" s="13">
         <v>340000</v>
@@ -2968,17 +2970,17 @@
       </c>
       <c r="B60">
         <f t="shared" si="0"/>
-        <v>5.0827788494037089E-4</v>
+        <v>0.33710580354050401</v>
       </c>
       <c r="C60">
         <f t="shared" si="3"/>
-        <v>0.99949172211505966</v>
+        <v>0.66289419645949599</v>
       </c>
       <c r="D60" s="5">
         <v>2023</v>
       </c>
       <c r="E60" s="12">
-        <v>620407945.47710001</v>
+        <v>620407.94547709997</v>
       </c>
       <c r="F60" s="6">
         <v>315500</v>
@@ -3011,24 +3013,24 @@
       </c>
       <c r="B61">
         <f t="shared" si="0"/>
-        <v>0.14485905299590882</v>
+        <v>0.99413138196173867</v>
       </c>
       <c r="C61">
         <f t="shared" si="3"/>
-        <v>0.85514094700409116</v>
+        <v>5.868618038261348E-3</v>
       </c>
       <c r="D61" s="5">
         <v>2024</v>
       </c>
       <c r="E61" s="12">
-        <v>830648000</v>
+        <v>830648</v>
       </c>
       <c r="F61" s="6">
         <v>140710000</v>
       </c>
       <c r="G61" s="6">
         <f>E61+F61</f>
-        <v>971358000</v>
+        <v>141540648</v>
       </c>
       <c r="H61" s="9">
         <v>382500</v>

</xml_diff>